<commit_message>
:fondue: adujst ASVs depth filter (150 for 16S, 250 for ITS) & ASVs prevalence filter (60%)
</commit_message>
<xml_diff>
--- a/data/derived_data/2_RarefyData/Dataset_1/ps_rare_ITS_sample_data_D1.xlsx
+++ b/data/derived_data/2_RarefyData/Dataset_1/ps_rare_ITS_sample_data_D1.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="236">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -501,6 +501,9 @@
   </si>
   <si>
     <t xml:space="preserve">MS_155</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_156</t>
   </si>
   <si>
     <t xml:space="preserve">MS_157</t>
@@ -6841,7 +6844,7 @@
         <v>151</v>
       </c>
       <c r="E99" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="F99" t="s">
         <v>152</v>
@@ -6859,19 +6862,19 @@
         <v>51</v>
       </c>
       <c r="K99" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="L99" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="M99" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="N99" t="s">
         <v>26</v>
       </c>
       <c r="O99" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="P99" t="s">
         <v>27</v>
@@ -6930,7 +6933,7 @@
         <v>26</v>
       </c>
       <c r="O100" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="P100" t="s">
         <v>27</v>
@@ -6989,7 +6992,7 @@
         <v>26</v>
       </c>
       <c r="O101" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="P101" t="s">
         <v>27</v>
@@ -7018,7 +7021,7 @@
         <v>151</v>
       </c>
       <c r="E102" t="s">
-        <v>57</v>
+        <v>22</v>
       </c>
       <c r="F102" t="s">
         <v>152</v>
@@ -7027,28 +7030,28 @@
         <v>24</v>
       </c>
       <c r="H102" t="s">
-        <v>25</v>
+        <v>66</v>
       </c>
       <c r="I102" t="s">
         <v>34</v>
       </c>
       <c r="J102" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="K102" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="L102" t="s">
-        <v>37</v>
+        <v>59</v>
       </c>
       <c r="M102" t="s">
-        <v>38</v>
+        <v>60</v>
       </c>
       <c r="N102" t="s">
         <v>26</v>
       </c>
       <c r="O102" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="P102" t="s">
         <v>27</v>
@@ -7107,7 +7110,7 @@
         <v>26</v>
       </c>
       <c r="O103" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="P103" t="s">
         <v>27</v>
@@ -7136,7 +7139,7 @@
         <v>151</v>
       </c>
       <c r="E104" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="F104" t="s">
         <v>152</v>
@@ -7166,7 +7169,7 @@
         <v>26</v>
       </c>
       <c r="O104" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="P104" t="s">
         <v>27</v>
@@ -7210,22 +7213,22 @@
         <v>34</v>
       </c>
       <c r="J105" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="K105" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="L105" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="M105" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="N105" t="s">
         <v>26</v>
       </c>
       <c r="O105" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="P105" t="s">
         <v>27</v>
@@ -7284,7 +7287,7 @@
         <v>26</v>
       </c>
       <c r="O106" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="P106" t="s">
         <v>27</v>
@@ -7313,7 +7316,7 @@
         <v>151</v>
       </c>
       <c r="E107" t="s">
-        <v>57</v>
+        <v>22</v>
       </c>
       <c r="F107" t="s">
         <v>152</v>
@@ -7343,7 +7346,7 @@
         <v>26</v>
       </c>
       <c r="O107" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="P107" t="s">
         <v>27</v>
@@ -7372,7 +7375,7 @@
         <v>151</v>
       </c>
       <c r="E108" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="F108" t="s">
         <v>152</v>
@@ -7393,16 +7396,16 @@
         <v>42</v>
       </c>
       <c r="L108" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="M108" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="N108" t="s">
         <v>26</v>
       </c>
       <c r="O108" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="P108" t="s">
         <v>27</v>
@@ -7431,7 +7434,7 @@
         <v>151</v>
       </c>
       <c r="E109" t="s">
-        <v>57</v>
+        <v>29</v>
       </c>
       <c r="F109" t="s">
         <v>152</v>
@@ -7461,7 +7464,7 @@
         <v>26</v>
       </c>
       <c r="O109" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="P109" t="s">
         <v>27</v>
@@ -7490,7 +7493,7 @@
         <v>151</v>
       </c>
       <c r="E110" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="F110" t="s">
         <v>152</v>
@@ -7505,22 +7508,22 @@
         <v>34</v>
       </c>
       <c r="J110" t="s">
+        <v>41</v>
+      </c>
+      <c r="K110" t="s">
+        <v>42</v>
+      </c>
+      <c r="L110" t="s">
+        <v>43</v>
+      </c>
+      <c r="M110" t="s">
+        <v>44</v>
+      </c>
+      <c r="N110" t="s">
+        <v>26</v>
+      </c>
+      <c r="O110" t="s">
         <v>51</v>
-      </c>
-      <c r="K110" t="s">
-        <v>52</v>
-      </c>
-      <c r="L110" t="s">
-        <v>53</v>
-      </c>
-      <c r="M110" t="s">
-        <v>54</v>
-      </c>
-      <c r="N110" t="s">
-        <v>26</v>
-      </c>
-      <c r="O110" t="s">
-        <v>35</v>
       </c>
       <c r="P110" t="s">
         <v>27</v>
@@ -7579,7 +7582,7 @@
         <v>26</v>
       </c>
       <c r="O111" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="P111" t="s">
         <v>27</v>
@@ -7638,7 +7641,7 @@
         <v>26</v>
       </c>
       <c r="O112" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="P112" t="s">
         <v>27</v>
@@ -7685,19 +7688,19 @@
         <v>51</v>
       </c>
       <c r="K113" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="L113" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="M113" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="N113" t="s">
         <v>26</v>
       </c>
       <c r="O113" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="P113" t="s">
         <v>27</v>
@@ -7756,7 +7759,7 @@
         <v>26</v>
       </c>
       <c r="O114" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="P114" t="s">
         <v>27</v>
@@ -7785,7 +7788,7 @@
         <v>151</v>
       </c>
       <c r="E115" t="s">
-        <v>57</v>
+        <v>22</v>
       </c>
       <c r="F115" t="s">
         <v>152</v>
@@ -7815,7 +7818,7 @@
         <v>26</v>
       </c>
       <c r="O115" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="P115" t="s">
         <v>27</v>
@@ -7838,52 +7841,52 @@
         <v>20</v>
       </c>
       <c r="C116" t="s">
-        <v>62</v>
+        <v>29</v>
       </c>
       <c r="D116" t="s">
-        <v>181</v>
+        <v>151</v>
       </c>
       <c r="E116" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="F116" t="s">
-        <v>182</v>
+        <v>152</v>
       </c>
       <c r="G116" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="H116" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I116" t="s">
         <v>34</v>
       </c>
       <c r="J116" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="K116" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="L116" t="s">
-        <v>37</v>
+        <v>59</v>
       </c>
       <c r="M116" t="s">
-        <v>38</v>
+        <v>60</v>
       </c>
       <c r="N116" t="s">
-        <v>183</v>
+        <v>26</v>
       </c>
       <c r="O116" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="P116" t="s">
         <v>27</v>
       </c>
       <c r="Q116" t="s">
-        <v>26</v>
+        <v>153</v>
       </c>
       <c r="R116" t="s">
-        <v>82</v>
+        <v>26</v>
       </c>
       <c r="S116" t="s">
         <v>180</v>
@@ -7891,22 +7894,22 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B117" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="C117" t="s">
         <v>62</v>
       </c>
       <c r="D117" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E117" t="s">
         <v>22</v>
       </c>
       <c r="F117" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G117" t="s">
         <v>33</v>
@@ -7930,7 +7933,7 @@
         <v>38</v>
       </c>
       <c r="N117" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="O117" t="s">
         <v>26</v>
@@ -7945,7 +7948,7 @@
         <v>82</v>
       </c>
       <c r="S117" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="118">
@@ -7953,19 +7956,19 @@
         <v>185</v>
       </c>
       <c r="B118" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="C118" t="s">
         <v>62</v>
       </c>
       <c r="D118" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E118" t="s">
         <v>22</v>
       </c>
       <c r="F118" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G118" t="s">
         <v>33</v>
@@ -7977,19 +7980,19 @@
         <v>34</v>
       </c>
       <c r="J118" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="K118" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="L118" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="M118" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="N118" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="O118" t="s">
         <v>26</v>
@@ -8012,19 +8015,19 @@
         <v>186</v>
       </c>
       <c r="B119" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="C119" t="s">
         <v>62</v>
       </c>
       <c r="D119" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E119" t="s">
         <v>22</v>
       </c>
       <c r="F119" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G119" t="s">
         <v>33</v>
@@ -8048,7 +8051,7 @@
         <v>48</v>
       </c>
       <c r="N119" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="O119" t="s">
         <v>26</v>
@@ -8071,19 +8074,19 @@
         <v>187</v>
       </c>
       <c r="B120" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="C120" t="s">
         <v>62</v>
       </c>
       <c r="D120" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E120" t="s">
         <v>22</v>
       </c>
       <c r="F120" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G120" t="s">
         <v>33</v>
@@ -8095,19 +8098,19 @@
         <v>34</v>
       </c>
       <c r="J120" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="K120" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="L120" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="M120" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="N120" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="O120" t="s">
         <v>26</v>
@@ -8130,19 +8133,19 @@
         <v>188</v>
       </c>
       <c r="B121" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="C121" t="s">
         <v>62</v>
       </c>
       <c r="D121" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E121" t="s">
         <v>22</v>
       </c>
       <c r="F121" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G121" t="s">
         <v>33</v>
@@ -8166,7 +8169,7 @@
         <v>54</v>
       </c>
       <c r="N121" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="O121" t="s">
         <v>26</v>
@@ -8189,19 +8192,19 @@
         <v>189</v>
       </c>
       <c r="B122" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="C122" t="s">
         <v>62</v>
       </c>
       <c r="D122" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E122" t="s">
         <v>22</v>
       </c>
       <c r="F122" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G122" t="s">
         <v>33</v>
@@ -8216,16 +8219,16 @@
         <v>51</v>
       </c>
       <c r="K122" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="L122" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="M122" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="N122" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="O122" t="s">
         <v>26</v>
@@ -8248,19 +8251,19 @@
         <v>190</v>
       </c>
       <c r="B123" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="C123" t="s">
         <v>62</v>
       </c>
       <c r="D123" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E123" t="s">
         <v>22</v>
       </c>
       <c r="F123" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G123" t="s">
         <v>33</v>
@@ -8284,7 +8287,7 @@
         <v>60</v>
       </c>
       <c r="N123" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="O123" t="s">
         <v>26</v>
@@ -8307,19 +8310,19 @@
         <v>191</v>
       </c>
       <c r="B124" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="C124" t="s">
         <v>62</v>
       </c>
       <c r="D124" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E124" t="s">
         <v>22</v>
       </c>
       <c r="F124" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G124" t="s">
         <v>33</v>
@@ -8331,19 +8334,19 @@
         <v>34</v>
       </c>
       <c r="J124" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="K124" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="L124" t="s">
-        <v>37</v>
+        <v>59</v>
       </c>
       <c r="M124" t="s">
-        <v>38</v>
+        <v>60</v>
       </c>
       <c r="N124" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="O124" t="s">
         <v>26</v>
@@ -8366,19 +8369,19 @@
         <v>192</v>
       </c>
       <c r="B125" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="C125" t="s">
         <v>62</v>
       </c>
       <c r="D125" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E125" t="s">
         <v>22</v>
       </c>
       <c r="F125" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G125" t="s">
         <v>33</v>
@@ -8402,7 +8405,7 @@
         <v>38</v>
       </c>
       <c r="N125" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="O125" t="s">
         <v>26</v>
@@ -8425,25 +8428,25 @@
         <v>193</v>
       </c>
       <c r="B126" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="C126" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
       <c r="D126" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="E126" t="s">
-        <v>62</v>
+        <v>22</v>
       </c>
       <c r="F126" t="s">
-        <v>195</v>
+        <v>183</v>
       </c>
       <c r="G126" t="s">
         <v>33</v>
       </c>
       <c r="H126" t="s">
-        <v>66</v>
+        <v>26</v>
       </c>
       <c r="I126" t="s">
         <v>34</v>
@@ -8461,19 +8464,19 @@
         <v>38</v>
       </c>
       <c r="N126" t="s">
-        <v>26</v>
+        <v>184</v>
       </c>
       <c r="O126" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="P126" t="s">
         <v>27</v>
       </c>
       <c r="Q126" t="s">
-        <v>195</v>
+        <v>26</v>
       </c>
       <c r="R126" t="s">
-        <v>26</v>
+        <v>82</v>
       </c>
       <c r="S126" t="s">
         <v>193</v>
@@ -8481,7 +8484,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B127" t="s">
         <v>20</v>
@@ -8490,13 +8493,13 @@
         <v>29</v>
       </c>
       <c r="D127" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E127" t="s">
         <v>62</v>
       </c>
       <c r="F127" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G127" t="s">
         <v>33</v>
@@ -8523,19 +8526,19 @@
         <v>26</v>
       </c>
       <c r="O127" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="P127" t="s">
         <v>27</v>
       </c>
       <c r="Q127" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R127" t="s">
         <v>26</v>
       </c>
       <c r="S127" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="128">
@@ -8549,13 +8552,13 @@
         <v>29</v>
       </c>
       <c r="D128" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E128" t="s">
         <v>62</v>
       </c>
       <c r="F128" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G128" t="s">
         <v>33</v>
@@ -8582,13 +8585,13 @@
         <v>26</v>
       </c>
       <c r="O128" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="P128" t="s">
         <v>27</v>
       </c>
       <c r="Q128" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R128" t="s">
         <v>26</v>
@@ -8608,13 +8611,13 @@
         <v>29</v>
       </c>
       <c r="D129" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E129" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="F129" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G129" t="s">
         <v>33</v>
@@ -8626,28 +8629,28 @@
         <v>34</v>
       </c>
       <c r="J129" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="K129" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="L129" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="M129" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="N129" t="s">
         <v>26</v>
       </c>
       <c r="O129" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="P129" t="s">
         <v>27</v>
       </c>
       <c r="Q129" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R129" t="s">
         <v>26</v>
@@ -8667,13 +8670,13 @@
         <v>29</v>
       </c>
       <c r="D130" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E130" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="F130" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G130" t="s">
         <v>33</v>
@@ -8700,13 +8703,13 @@
         <v>26</v>
       </c>
       <c r="O130" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="P130" t="s">
         <v>27</v>
       </c>
       <c r="Q130" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R130" t="s">
         <v>26</v>
@@ -8726,13 +8729,13 @@
         <v>29</v>
       </c>
       <c r="D131" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E131" t="s">
         <v>22</v>
       </c>
       <c r="F131" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G131" t="s">
         <v>33</v>
@@ -8759,13 +8762,13 @@
         <v>26</v>
       </c>
       <c r="O131" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="P131" t="s">
         <v>27</v>
       </c>
       <c r="Q131" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R131" t="s">
         <v>26</v>
@@ -8785,13 +8788,13 @@
         <v>29</v>
       </c>
       <c r="D132" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E132" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F132" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G132" t="s">
         <v>33</v>
@@ -8809,22 +8812,22 @@
         <v>42</v>
       </c>
       <c r="L132" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="M132" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="N132" t="s">
         <v>26</v>
       </c>
       <c r="O132" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="P132" t="s">
         <v>27</v>
       </c>
       <c r="Q132" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R132" t="s">
         <v>26</v>
@@ -8844,13 +8847,13 @@
         <v>29</v>
       </c>
       <c r="D133" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E133" t="s">
-        <v>62</v>
+        <v>29</v>
       </c>
       <c r="F133" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G133" t="s">
         <v>33</v>
@@ -8877,13 +8880,13 @@
         <v>26</v>
       </c>
       <c r="O133" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="P133" t="s">
         <v>27</v>
       </c>
       <c r="Q133" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R133" t="s">
         <v>26</v>
@@ -8903,13 +8906,13 @@
         <v>29</v>
       </c>
       <c r="D134" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E134" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
       <c r="F134" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G134" t="s">
         <v>33</v>
@@ -8936,13 +8939,13 @@
         <v>26</v>
       </c>
       <c r="O134" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="P134" t="s">
         <v>27</v>
       </c>
       <c r="Q134" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R134" t="s">
         <v>26</v>
@@ -8962,13 +8965,13 @@
         <v>29</v>
       </c>
       <c r="D135" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E135" t="s">
         <v>29</v>
       </c>
       <c r="F135" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G135" t="s">
         <v>33</v>
@@ -8980,28 +8983,28 @@
         <v>34</v>
       </c>
       <c r="J135" t="s">
+        <v>41</v>
+      </c>
+      <c r="K135" t="s">
+        <v>42</v>
+      </c>
+      <c r="L135" t="s">
+        <v>43</v>
+      </c>
+      <c r="M135" t="s">
+        <v>44</v>
+      </c>
+      <c r="N135" t="s">
+        <v>26</v>
+      </c>
+      <c r="O135" t="s">
         <v>51</v>
       </c>
-      <c r="K135" t="s">
-        <v>52</v>
-      </c>
-      <c r="L135" t="s">
-        <v>53</v>
-      </c>
-      <c r="M135" t="s">
-        <v>54</v>
-      </c>
-      <c r="N135" t="s">
-        <v>26</v>
-      </c>
-      <c r="O135" t="s">
-        <v>35</v>
-      </c>
       <c r="P135" t="s">
         <v>27</v>
       </c>
       <c r="Q135" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R135" t="s">
         <v>26</v>
@@ -9021,13 +9024,13 @@
         <v>29</v>
       </c>
       <c r="D136" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E136" t="s">
         <v>29</v>
       </c>
       <c r="F136" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G136" t="s">
         <v>33</v>
@@ -9054,13 +9057,13 @@
         <v>26</v>
       </c>
       <c r="O136" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="P136" t="s">
         <v>27</v>
       </c>
       <c r="Q136" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R136" t="s">
         <v>26</v>
@@ -9080,13 +9083,13 @@
         <v>29</v>
       </c>
       <c r="D137" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E137" t="s">
-        <v>57</v>
+        <v>29</v>
       </c>
       <c r="F137" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G137" t="s">
         <v>33</v>
@@ -9113,13 +9116,13 @@
         <v>26</v>
       </c>
       <c r="O137" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="P137" t="s">
         <v>27</v>
       </c>
       <c r="Q137" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R137" t="s">
         <v>26</v>
@@ -9139,13 +9142,13 @@
         <v>29</v>
       </c>
       <c r="D138" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E138" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="F138" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G138" t="s">
         <v>33</v>
@@ -9160,25 +9163,25 @@
         <v>51</v>
       </c>
       <c r="K138" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="L138" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="M138" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="N138" t="s">
         <v>26</v>
       </c>
       <c r="O138" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="P138" t="s">
         <v>27</v>
       </c>
       <c r="Q138" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R138" t="s">
         <v>26</v>
@@ -9198,13 +9201,13 @@
         <v>29</v>
       </c>
       <c r="D139" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E139" t="s">
         <v>22</v>
       </c>
       <c r="F139" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G139" t="s">
         <v>33</v>
@@ -9231,13 +9234,13 @@
         <v>26</v>
       </c>
       <c r="O139" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="P139" t="s">
         <v>27</v>
       </c>
       <c r="Q139" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R139" t="s">
         <v>26</v>
@@ -9257,13 +9260,13 @@
         <v>29</v>
       </c>
       <c r="D140" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E140" t="s">
         <v>22</v>
       </c>
       <c r="F140" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G140" t="s">
         <v>33</v>
@@ -9290,13 +9293,13 @@
         <v>26</v>
       </c>
       <c r="O140" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="P140" t="s">
         <v>27</v>
       </c>
       <c r="Q140" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R140" t="s">
         <v>26</v>
@@ -9316,46 +9319,46 @@
         <v>29</v>
       </c>
       <c r="D141" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E141" t="s">
-        <v>57</v>
+        <v>22</v>
       </c>
       <c r="F141" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G141" t="s">
         <v>33</v>
       </c>
       <c r="H141" t="s">
-        <v>25</v>
+        <v>66</v>
       </c>
       <c r="I141" t="s">
         <v>34</v>
       </c>
       <c r="J141" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="K141" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="L141" t="s">
-        <v>37</v>
+        <v>59</v>
       </c>
       <c r="M141" t="s">
-        <v>38</v>
+        <v>60</v>
       </c>
       <c r="N141" t="s">
         <v>26</v>
       </c>
       <c r="O141" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="P141" t="s">
         <v>27</v>
       </c>
       <c r="Q141" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R141" t="s">
         <v>26</v>
@@ -9375,13 +9378,13 @@
         <v>29</v>
       </c>
       <c r="D142" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E142" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="F142" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G142" t="s">
         <v>33</v>
@@ -9408,13 +9411,13 @@
         <v>26</v>
       </c>
       <c r="O142" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="P142" t="s">
         <v>27</v>
       </c>
       <c r="Q142" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R142" t="s">
         <v>26</v>
@@ -9434,13 +9437,13 @@
         <v>29</v>
       </c>
       <c r="D143" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E143" t="s">
-        <v>57</v>
+        <v>22</v>
       </c>
       <c r="F143" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G143" t="s">
         <v>33</v>
@@ -9452,28 +9455,28 @@
         <v>34</v>
       </c>
       <c r="J143" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="K143" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="L143" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="M143" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="N143" t="s">
         <v>26</v>
       </c>
       <c r="O143" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="P143" t="s">
         <v>27</v>
       </c>
       <c r="Q143" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R143" t="s">
         <v>26</v>
@@ -9493,13 +9496,13 @@
         <v>29</v>
       </c>
       <c r="D144" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E144" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="F144" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G144" t="s">
         <v>33</v>
@@ -9526,13 +9529,13 @@
         <v>26</v>
       </c>
       <c r="O144" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="P144" t="s">
         <v>27</v>
       </c>
       <c r="Q144" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R144" t="s">
         <v>26</v>
@@ -9552,13 +9555,13 @@
         <v>29</v>
       </c>
       <c r="D145" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E145" t="s">
-        <v>57</v>
+        <v>22</v>
       </c>
       <c r="F145" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G145" t="s">
         <v>33</v>
@@ -9585,13 +9588,13 @@
         <v>26</v>
       </c>
       <c r="O145" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="P145" t="s">
         <v>27</v>
       </c>
       <c r="Q145" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R145" t="s">
         <v>26</v>
@@ -9611,13 +9614,13 @@
         <v>29</v>
       </c>
       <c r="D146" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E146" t="s">
         <v>57</v>
       </c>
       <c r="F146" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G146" t="s">
         <v>33</v>
@@ -9635,22 +9638,22 @@
         <v>42</v>
       </c>
       <c r="L146" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="M146" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="N146" t="s">
         <v>26</v>
       </c>
       <c r="O146" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="P146" t="s">
         <v>27</v>
       </c>
       <c r="Q146" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R146" t="s">
         <v>26</v>
@@ -9670,13 +9673,13 @@
         <v>29</v>
       </c>
       <c r="D147" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E147" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="F147" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G147" t="s">
         <v>33</v>
@@ -9703,13 +9706,13 @@
         <v>26</v>
       </c>
       <c r="O147" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="P147" t="s">
         <v>27</v>
       </c>
       <c r="Q147" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R147" t="s">
         <v>26</v>
@@ -9729,13 +9732,13 @@
         <v>29</v>
       </c>
       <c r="D148" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E148" t="s">
-        <v>57</v>
+        <v>29</v>
       </c>
       <c r="F148" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G148" t="s">
         <v>33</v>
@@ -9762,13 +9765,13 @@
         <v>26</v>
       </c>
       <c r="O148" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="P148" t="s">
         <v>27</v>
       </c>
       <c r="Q148" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R148" t="s">
         <v>26</v>
@@ -9788,13 +9791,13 @@
         <v>29</v>
       </c>
       <c r="D149" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E149" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="F149" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G149" t="s">
         <v>33</v>
@@ -9806,28 +9809,28 @@
         <v>34</v>
       </c>
       <c r="J149" t="s">
+        <v>41</v>
+      </c>
+      <c r="K149" t="s">
+        <v>42</v>
+      </c>
+      <c r="L149" t="s">
+        <v>43</v>
+      </c>
+      <c r="M149" t="s">
+        <v>44</v>
+      </c>
+      <c r="N149" t="s">
+        <v>26</v>
+      </c>
+      <c r="O149" t="s">
         <v>51</v>
       </c>
-      <c r="K149" t="s">
-        <v>52</v>
-      </c>
-      <c r="L149" t="s">
-        <v>53</v>
-      </c>
-      <c r="M149" t="s">
-        <v>54</v>
-      </c>
-      <c r="N149" t="s">
-        <v>26</v>
-      </c>
-      <c r="O149" t="s">
-        <v>41</v>
-      </c>
       <c r="P149" t="s">
         <v>27</v>
       </c>
       <c r="Q149" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R149" t="s">
         <v>26</v>
@@ -9847,13 +9850,13 @@
         <v>29</v>
       </c>
       <c r="D150" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E150" t="s">
         <v>22</v>
       </c>
       <c r="F150" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G150" t="s">
         <v>33</v>
@@ -9880,13 +9883,13 @@
         <v>26</v>
       </c>
       <c r="O150" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="P150" t="s">
         <v>27</v>
       </c>
       <c r="Q150" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R150" t="s">
         <v>26</v>
@@ -9906,13 +9909,13 @@
         <v>29</v>
       </c>
       <c r="D151" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E151" t="s">
         <v>22</v>
       </c>
       <c r="F151" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G151" t="s">
         <v>33</v>
@@ -9927,25 +9930,25 @@
         <v>51</v>
       </c>
       <c r="K151" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="L151" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="M151" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="N151" t="s">
         <v>26</v>
       </c>
       <c r="O151" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="P151" t="s">
         <v>27</v>
       </c>
       <c r="Q151" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R151" t="s">
         <v>26</v>
@@ -9965,13 +9968,13 @@
         <v>29</v>
       </c>
       <c r="D152" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E152" t="s">
         <v>22</v>
       </c>
       <c r="F152" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G152" t="s">
         <v>33</v>
@@ -9998,13 +10001,13 @@
         <v>26</v>
       </c>
       <c r="O152" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="P152" t="s">
         <v>27</v>
       </c>
       <c r="Q152" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R152" t="s">
         <v>26</v>
@@ -10024,13 +10027,13 @@
         <v>29</v>
       </c>
       <c r="D153" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E153" t="s">
-        <v>57</v>
+        <v>22</v>
       </c>
       <c r="F153" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G153" t="s">
         <v>33</v>
@@ -10057,13 +10060,13 @@
         <v>26</v>
       </c>
       <c r="O153" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="P153" t="s">
         <v>27</v>
       </c>
       <c r="Q153" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R153" t="s">
         <v>26</v>
@@ -10080,52 +10083,52 @@
         <v>20</v>
       </c>
       <c r="C154" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="D154" t="s">
-        <v>21</v>
+        <v>195</v>
       </c>
       <c r="E154" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="F154" t="s">
-        <v>224</v>
+        <v>196</v>
       </c>
       <c r="G154" t="s">
-        <v>225</v>
+        <v>33</v>
       </c>
       <c r="H154" t="s">
         <v>25</v>
       </c>
       <c r="I154" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="J154" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="K154" t="s">
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="L154" t="s">
-        <v>26</v>
+        <v>59</v>
       </c>
       <c r="M154" t="s">
-        <v>26</v>
+        <v>60</v>
       </c>
       <c r="N154" t="s">
         <v>26</v>
       </c>
       <c r="O154" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="P154" t="s">
         <v>27</v>
       </c>
       <c r="Q154" t="s">
-        <v>26</v>
+        <v>196</v>
       </c>
       <c r="R154" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="S154" t="s">
         <v>223</v>
@@ -10133,10 +10136,10 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B155" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="C155" t="s">
         <v>20</v>
@@ -10148,10 +10151,10 @@
         <v>22</v>
       </c>
       <c r="F155" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="G155" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="H155" t="s">
         <v>25</v>
@@ -10187,7 +10190,7 @@
         <v>23</v>
       </c>
       <c r="S155" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="156">
@@ -10195,40 +10198,40 @@
         <v>227</v>
       </c>
       <c r="B156" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="C156" t="s">
         <v>20</v>
       </c>
       <c r="D156" t="s">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="E156" t="s">
-        <v>62</v>
+        <v>22</v>
       </c>
       <c r="F156" t="s">
-        <v>65</v>
+        <v>225</v>
       </c>
       <c r="G156" t="s">
-        <v>24</v>
+        <v>226</v>
       </c>
       <c r="H156" t="s">
-        <v>66</v>
+        <v>25</v>
       </c>
       <c r="I156" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="J156" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="K156" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="L156" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="M156" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="N156" t="s">
         <v>26</v>
@@ -10240,10 +10243,10 @@
         <v>27</v>
       </c>
       <c r="Q156" t="s">
-        <v>65</v>
+        <v>26</v>
       </c>
       <c r="R156" t="s">
-        <v>65</v>
+        <v>23</v>
       </c>
       <c r="S156" t="s">
         <v>227</v>
@@ -10278,16 +10281,16 @@
         <v>34</v>
       </c>
       <c r="J157" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="K157" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="L157" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="M157" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="N157" t="s">
         <v>26</v>
@@ -10322,7 +10325,7 @@
         <v>64</v>
       </c>
       <c r="E158" t="s">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="F158" t="s">
         <v>65</v>
@@ -10337,16 +10340,16 @@
         <v>34</v>
       </c>
       <c r="J158" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="K158" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="L158" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="M158" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="N158" t="s">
         <v>26</v>
@@ -10381,7 +10384,7 @@
         <v>64</v>
       </c>
       <c r="E159" t="s">
-        <v>62</v>
+        <v>22</v>
       </c>
       <c r="F159" t="s">
         <v>65</v>
@@ -10399,13 +10402,13 @@
         <v>51</v>
       </c>
       <c r="K159" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="L159" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="M159" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="N159" t="s">
         <v>26</v>
@@ -10440,7 +10443,7 @@
         <v>64</v>
       </c>
       <c r="E160" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
       <c r="F160" t="s">
         <v>65</v>
@@ -10449,22 +10452,22 @@
         <v>24</v>
       </c>
       <c r="H160" t="s">
-        <v>25</v>
+        <v>66</v>
       </c>
       <c r="I160" t="s">
         <v>34</v>
       </c>
       <c r="J160" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="K160" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="L160" t="s">
-        <v>37</v>
+        <v>59</v>
       </c>
       <c r="M160" t="s">
-        <v>38</v>
+        <v>60</v>
       </c>
       <c r="N160" t="s">
         <v>26</v>
@@ -10514,16 +10517,16 @@
         <v>34</v>
       </c>
       <c r="J161" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="K161" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="L161" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="M161" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="N161" t="s">
         <v>26</v>
@@ -10558,7 +10561,7 @@
         <v>64</v>
       </c>
       <c r="E162" t="s">
-        <v>62</v>
+        <v>29</v>
       </c>
       <c r="F162" t="s">
         <v>65</v>
@@ -10573,16 +10576,16 @@
         <v>34</v>
       </c>
       <c r="J162" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="K162" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="L162" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="M162" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="N162" t="s">
         <v>26</v>
@@ -10617,7 +10620,7 @@
         <v>64</v>
       </c>
       <c r="E163" t="s">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="F163" t="s">
         <v>65</v>
@@ -10632,16 +10635,16 @@
         <v>34</v>
       </c>
       <c r="J163" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="K163" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="L163" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="M163" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="N163" t="s">
         <v>26</v>
@@ -10660,6 +10663,65 @@
       </c>
       <c r="S163" t="s">
         <v>234</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="s">
+        <v>235</v>
+      </c>
+      <c r="B164" t="s">
+        <v>20</v>
+      </c>
+      <c r="C164" t="s">
+        <v>20</v>
+      </c>
+      <c r="D164" t="s">
+        <v>64</v>
+      </c>
+      <c r="E164" t="s">
+        <v>22</v>
+      </c>
+      <c r="F164" t="s">
+        <v>65</v>
+      </c>
+      <c r="G164" t="s">
+        <v>24</v>
+      </c>
+      <c r="H164" t="s">
+        <v>25</v>
+      </c>
+      <c r="I164" t="s">
+        <v>34</v>
+      </c>
+      <c r="J164" t="s">
+        <v>51</v>
+      </c>
+      <c r="K164" t="s">
+        <v>58</v>
+      </c>
+      <c r="L164" t="s">
+        <v>59</v>
+      </c>
+      <c r="M164" t="s">
+        <v>60</v>
+      </c>
+      <c r="N164" t="s">
+        <v>26</v>
+      </c>
+      <c r="O164" t="s">
+        <v>26</v>
+      </c>
+      <c r="P164" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q164" t="s">
+        <v>65</v>
+      </c>
+      <c r="R164" t="s">
+        <v>65</v>
+      </c>
+      <c r="S164" t="s">
+        <v>235</v>
       </c>
     </row>
   </sheetData>

</xml_diff>